<commit_message>
Ask DOLD for igus drag chains and MR12 carriages
Dold Bestellung.xlsx gets a separate section with the parts so far
planned at igus and Motedis (8 + 8 drag chains, 12 MR12 carriages),
so DOLD can check whether they can supply them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/Dold Bestellung.xlsx
+++ b/bom/Dold Bestellung.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -443,6 +443,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -460,6 +461,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1189,6 +1191,58 @@
       <c r="C56" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-125-Form-A-Unterlegscheibe-Stahl-verzinkt-d53mm-D10mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Zusätzlich anfragen – bisher bei igus / Motedis geplant (bitte prüfen, ob DOLD das liefern kann)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Linearwagen MR12 MN-SS-V0-N (bisher Motedis)</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>12</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://www.motedis.com/shop/Dynamik-Lineareinheiten/Profilschienenfuehrungen-fuer-die-Linearbewegung/Profilschienenfuehrungen/Fuehrungswagen-Miniatur-MR12MN-SS-V0-N::6097.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Energiekette igus E2i.10.20.028.0 (X), 14 Glieder = 0,28 m, inkl. Anschlussset E2.100.20.34PZ.A2 (bisher igus)</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>8</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://www.igus.de/product/series-E2i-10?artnr=E2I.10.20.028.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Energiekette igus E2i.10.10.028.0 (Y), 12 Glieder = 0,24 m, inkl. Anschlussset E2.100.10.34PZ.A2 (bisher igus)</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>8</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://www.igus.de/product/series-E2i-10?artnr=E2i.10.10.028.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update DOLD order list, rename Bestellliste to Bauteilliste, add tooled parts STEP
- Move MR12 600 mm rails and carriages to DOLD; drop M8 nuts (included with sensors)
- Set screw/nut quantities from CAD count plus reserve; small quantities from Werkstatt
- Add docs/offene-fragen.md and STEP export of all parts to be machined

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/Dold Bestellung.xlsx
+++ b/bom/Dold Bestellung.xlsx
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -852,11 +852,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M3x12, A2</t>
+          <t>DIN 912 (ISO 4762) Zylinderschraube M3x16, A2</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -867,11 +867,11 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M3x14, A2</t>
+          <t>DIN 912 (ISO 4762) Zylinderschraube M3x18, A2</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -882,7 +882,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M3x16, A2</t>
+          <t>DIN 912 (ISO 4762) Zylinderschraube M4x20, A2</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -897,11 +897,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M3x18, A2</t>
+          <t>DIN 912 (ISO 4762) Zylinderschraube M4x30, A2</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -912,11 +912,11 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M3x20, A2</t>
+          <t>DIN 912 (ISO 4762) Zylinderschraube M5x10, A2</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -927,320 +927,170 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M3x30, A2</t>
+          <t>DIN 7991 (ISO 10642) Senkschraube M3x8, A2</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+          <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M4x10, A2</t>
+          <t>DIN 7991 (ISO 10642) Senkschraube M6x12, A2</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+          <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M4x20, A2</t>
+          <t>DIN 7991 (ISO 10642) Senkschraube M6x20, A2</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+          <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M4x30, A2</t>
+          <t>DIN 934 (ISO 4032) Sechskantmutter M3, verzinkt</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+          <t>https://www.dold-mechatronik.de/DIN-934-Sechskantmutter-.8-verzinkt-M4x07</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M5x10, A2</t>
+          <t>DIN 934 (ISO 4032) Sechskantmutter M4, verzinkt</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>36</v>
+        <v>71</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+          <t>https://www.dold-mechatronik.de/DIN-934-Sechskantmutter-.8-verzinkt-M4x07</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DIN 912 (ISO 4762) Zylinderschraube M5x14, 8.8 verzinkt</t>
+          <t>Nutenstein Nut6, M5</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant-8.8-verzinkt</t>
+          <t>https://www.dold-mechatronik.de/Nutenstein-mit-Steg-I-Typ-Nut-6-Gewindedurchmesser-M5</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>DIN 7991 (ISO 10642) Senkschraube M3x8, A2</t>
+          <t>Nutenstein Nut6, M3</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
+          <t>https://www.dold-mechatronik.de/Nutenstein-mit-Steg-I-Typ-Nut-6-Gewindedurchmesser-M3</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DIN 7991 (ISO 10642) Senkschraube M6x12, A2</t>
+          <t>Unterlegscheiben M5</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>DIN 7991 (ISO 10642) Senkschraube M6x14, A2</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>8</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
+          <t>https://www.dold-mechatronik.de/DIN-125-Form-A-Unterlegscheibe-Stahl-verzinkt-d53mm-D10mm</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>DIN 7991 (ISO 10642) Senkschraube M6x20, A2</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>25</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Separat – bitte prüfen, was DOLD davon liefern kann (bisher bei igus / Motedis geplant)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DIN 933 (ISO 4017) Sechskantschraube M4x20, A2</t>
+          <t>Linearwagen MR12 MN-SS-V0-N, Blockmodell, Vorspannung V0, Genauigkeit N (Ihr Angebot AN2026-104489, Pos. 19/38)</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://www.dold-mechatronik.de/DIN-933-A2-Edelstahl-Sechskantschraube-mit-Gewinde-bis-Kopf.-Ausfuehrung-waehlbar</t>
+          <t>Art.-Nr. MR12 MN-SS-V0-N-BLOCK – 12 Stück statt 3 im Angebot, bitte Preis für diese Menge prüfen</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DIN 934 (ISO 4032) Sechskantmutter M3, verzinkt</t>
+          <t>Energiekette igus E2i.10.20.028.0 (X), 14 Glieder = 0,28 m, inkl. Anschlussset E2.100.20.34PZ.A2 (bisher igus)</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://www.dold-mechatronik.de/DIN-934-Sechskantmutter-.8-verzinkt-M4x07</t>
+          <t>https://www.igus.de/product/series-E2i-10?artnr=E2I.10.20.028.0</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DIN 934 (ISO 4032) Sechskantmutter M4, verzinkt</t>
+          <t>Energiekette igus E2i.10.10.028.0 (Y), 12 Glieder = 0,24 m, inkl. Anschlussset E2.100.10.34PZ.A2 (bisher igus)</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="C51" t="inlineStr">
-        <is>
-          <t>https://www.dold-mechatronik.de/DIN-934-Sechskantmutter-.8-verzinkt-M4x07</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>DIN 934 (ISO 4032) Sechskantmutter M8, A2</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>53</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>https://www.dold-mechatronik.de/Sechskantmutter-DIN-934-ISO-4032-M8-Edelstahl-A2</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>DIN 466 Rändelmutter hoch M4</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>10</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>https://www.dold-mechatronik.de/Hohe-Raendelmutter-Material-und-Groesse-waehlbar-NEU</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Nutenstein Nut6, M5</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>10</v>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>https://www.dold-mechatronik.de/Nutenstein-mit-Steg-I-Typ-Nut-6-Gewindedurchmesser-M5</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Nutenstein Nut6, M3</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>46</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>https://www.dold-mechatronik.de/Nutenstein-mit-Steg-I-Typ-Nut-6-Gewindedurchmesser-M3</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Unterlegscheiben M5</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>16</v>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>https://www.dold-mechatronik.de/DIN-125-Form-A-Unterlegscheibe-Stahl-verzinkt-d53mm-D10mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>Zusätzlich anfragen – bisher bei igus / Motedis geplant (bitte prüfen, ob DOLD das liefern kann)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Linearwagen MR12 MN-SS-V0-N (bisher Motedis)</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>12</v>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>https://www.motedis.com/shop/Dynamik-Lineareinheiten/Profilschienenfuehrungen-fuer-die-Linearbewegung/Profilschienenfuehrungen/Fuehrungswagen-Miniatur-MR12MN-SS-V0-N::6097.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Energiekette igus E2i.10.20.028.0 (X), 14 Glieder = 0,28 m, inkl. Anschlussset E2.100.20.34PZ.A2 (bisher igus)</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>8</v>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>https://www.igus.de/product/series-E2i-10?artnr=E2I.10.20.028.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Energiekette igus E2i.10.10.028.0 (Y), 12 Glieder = 0,24 m, inkl. Anschlussset E2.100.10.34PZ.A2 (bisher igus)</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>8</v>
-      </c>
-      <c r="C61" t="inlineStr">
         <is>
           <t>https://www.igus.de/product/series-E2i-10?artnr=E2i.10.10.028.0</t>
         </is>

</xml_diff>